<commit_message>
feat: 3D viewer integrated, BOM filtered by SVG intersection, Excel auto-watch
</commit_message>
<xml_diff>
--- a/resources/excel/ER5215-301.xlsx
+++ b/resources/excel/ER5215-301.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ER5215-301_DEV\resources\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SDTD-2\ER5215-301_DEV\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE234BB9-FBF6-4EE3-B07D-033579FB2314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08460343-8290-4867-9F05-71E4D387C403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>part_number</t>
   </si>
@@ -31,6 +31,33 @@
     <t>quantity</t>
   </si>
   <si>
+    <t>visible3d</t>
+  </si>
+  <si>
+    <t>905001</t>
+  </si>
+  <si>
+    <t>REDUCTEUR DODGE SMR TA5215H25</t>
+  </si>
+  <si>
+    <t>905022</t>
+  </si>
+  <si>
+    <t>MOYEU 2 15/16" SMR TA5215TB</t>
+  </si>
+  <si>
+    <t>905102</t>
+  </si>
+  <si>
+    <t>ANTI-RECUL DODGE TA5215BS</t>
+  </si>
+  <si>
+    <t>905109</t>
+  </si>
+  <si>
+    <t>TA5215RA ROD ASSEMBLY</t>
+  </si>
+  <si>
     <t>AR112-037</t>
   </si>
   <si>
@@ -149,37 +176,13 @@
   </si>
   <si>
     <t>HUILE SYNTGEAR MOBIL SHC 629</t>
-  </si>
-  <si>
-    <t>905001</t>
-  </si>
-  <si>
-    <t>REDUCTEUR DODGE SMR TA5215H25</t>
-  </si>
-  <si>
-    <t>905022</t>
-  </si>
-  <si>
-    <t>MOYEU 2 15/16" SMR TA5215TB</t>
-  </si>
-  <si>
-    <t>905102</t>
-  </si>
-  <si>
-    <t>ANTI-RECUL DODGE TA5215BS</t>
-  </si>
-  <si>
-    <t>905109</t>
-  </si>
-  <si>
-    <t>TA5215RA ROD ASSEMBLY</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,8 +196,14 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,6 +213,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF005A9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -219,10 +234,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -239,6 +265,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -526,15 +569,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -544,275 +587,347 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="C11">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C13">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C14">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C15">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C16">
         <v>6</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C17">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C18">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C19">
         <v>6</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B21" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B22" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D22" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D23" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C24">
         <v>4</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D24" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C25">
         <v>7</v>
       </c>
+      <c r="D25" s="3" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C25">
-    <sortCondition ref="A2:A25"/>
-  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>